<commit_message>
Daily EOD data and reports for 2026-08-17
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260817.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260817.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.575</v>
+        <v>1.587</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.04</v>
+        <v>0.052</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>241260.07</v>
+        <v>243098.25</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>6127.24</v>
+        <v>7965.41</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.29</v>
+        <v>2.28</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.72%</t>
+          <t>-2.15%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>160300</v>
+        <v>159600</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-2800</v>
+        <v>-3500</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.24</v>
+        <v>1.245</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>2.05%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>71247.92</v>
+        <v>71535.21000000001</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>1149.16</v>
+        <v>1436.45</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>61.94</v>
+        <v>62.02</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.59</v>
+        <v>0.67</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>685366.1</v>
+        <v>686251.3</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>6528.35</v>
+        <v>7413.55</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>167.55</v>
+        <v>167.4</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.38</v>
+        <v>0.23</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.14%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.88</v>
+        <v>0.895</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.015</v>
+        <v>0.03</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.73%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>8800</v>
+        <v>8950</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>136.73</v>
+        <v>136.33</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.23</v>
+        <v>-0.17</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>546920</v>
+        <v>545320</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>920</v>
+        <v>-680</v>
       </c>
     </row>
     <row r="12">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.12</v>
+        <v>0.125</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1129.44</v>
+        <v>1176.5</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>47.06</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.45</v>
+        <v>35.25</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.08</v>
+        <v>-0.12</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>-0.34%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.795</v>
+        <v>32.985</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.195</v>
+        <v>0.385</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.60%</t>
+          <t>1.18%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42239.96</v>
+        <v>42484.68</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>251.16</v>
+        <v>495.88</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1763469.85</v>
+        <v>1764622.3</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>11200</v>
+        <v>12352.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>